<commit_message>
commit update aula 03062023
</commit_message>
<xml_diff>
--- a/Primeiro dia de Excel Avançado 03062023 - Yuri Mendes/ex_FAvançado.xlsx
+++ b/Primeiro dia de Excel Avançado 03062023 - Yuri Mendes/ex_FAvançado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noturno\Desktop\Excel Avançado - 2019 - Green - VAZIA\Exercícios Propostos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuri.smendes\Documents\Primeiro dia de Excel Avançado 03062023 - Yuri Mendes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5FA06E-45CC-4DC9-A0D2-F757356AD67B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94ECBBAA-F06D-41CC-B5FC-C7BF3A0AF531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="630" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="630" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Filtro Avançado 1" sheetId="4" r:id="rId1"/>
@@ -29,16 +29,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Filtro Avançado 4'!$A$1:$G$45</definedName>
     <definedName name="a" hidden="1">{"normal","argentina",FALSE,"cenários e solver";#N/A,#N/A,FALSE,"banco de dados"}</definedName>
     <definedName name="anscount" hidden="1">2</definedName>
-    <definedName name="_xlnm.Extract" localSheetId="0">'Filtro Avançado 1'!$I$12:$O$12</definedName>
-    <definedName name="_xlnm.Extract" localSheetId="1">'Filtro Avançado 2'!$I$7:$O$7</definedName>
-    <definedName name="_xlnm.Extract" localSheetId="2">'Filtro Avançado 3'!$I$9:$O$9</definedName>
-    <definedName name="_xlnm.Extract" localSheetId="3">'Filtro Avançado 4'!$I$9:$O$9</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="0">'Filtro Avançado 1'!$I$8:$O$8</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="1">'Filtro Avançado 2'!$I$9:$O$9</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="2">'Filtro Avançado 3'!$I$11:$O$11</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="3">'Filtro Avançado 4'!$I$13:$O$13</definedName>
     <definedName name="b" hidden="1">{"azul",#N/A,FALSE,"geral";"verde",#N/A,FALSE,"geral";"vermelho",#N/A,FALSE,"geral"}</definedName>
     <definedName name="conf" hidden="1">{"azul",#N/A,FALSE,"geral";"verde",#N/A,FALSE,"geral";"vermelho",#N/A,FALSE,"geral"}</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="0">'Filtro Avançado 1'!$I$7:$K$8</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="1">'Filtro Avançado 2'!$I$4:$K$5</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="2">'Filtro Avançado 3'!$I$4:$K$6</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="3">'Filtro Avançado 4'!$I$4:$L$6</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="0">'Filtro Avançado 1'!$I$5:$K$6</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="1">'Filtro Avançado 2'!$I$6:$K$7</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="2">'Filtro Avançado 3'!$I$7:$K$9</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="3">'Filtro Avançado 4'!$I$9:$L$11</definedName>
     <definedName name="d" hidden="1">{"azul",#N/A,FALSE,"geral";"verde",#N/A,FALSE,"geral";"vermelho",#N/A,FALSE,"geral"}</definedName>
     <definedName name="e" hidden="1">{"azul",#N/A,FALSE,"geral";"verde",#N/A,FALSE,"geral";"vermelho",#N/A,FALSE,"geral"}</definedName>
     <definedName name="Fev">'[1]4-Nomear Colunas'!$B$2:$B$10</definedName>
@@ -89,11 +89,24 @@
     <definedName name="yu" hidden="1">{"normal","argentina",FALSE,"cenários e solver";#N/A,#N/A,FALSE,"banco de dados"}</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="25">
   <si>
     <t>Data</t>
   </si>
@@ -165,6 +178,9 @@
   </si>
   <si>
     <t>Violino</t>
+  </si>
+  <si>
+    <t>&gt;3</t>
   </si>
 </sst>
 </file>
@@ -293,7 +309,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -307,6 +323,25 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -627,7 +662,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="4-Nomear Colunas"/>
@@ -767,7 +802,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="1-Relatório Geral"/>
@@ -1235,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -1245,7 +1280,7 @@
     <col min="6" max="7" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1268,7 +1303,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>33610</v>
       </c>
@@ -1292,7 +1327,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>33611</v>
       </c>
@@ -1316,7 +1351,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>33612</v>
       </c>
@@ -1340,7 +1375,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>33615</v>
       </c>
@@ -1363,8 +1398,17 @@
         <f t="shared" si="0"/>
         <v>3500</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>33616</v>
       </c>
@@ -1387,8 +1431,17 @@
         <f t="shared" si="0"/>
         <v>4980</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>33617</v>
       </c>
@@ -1412,7 +1465,7 @@
         <v>2240</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>33618</v>
       </c>
@@ -1435,8 +1488,29 @@
         <f t="shared" si="0"/>
         <v>3750</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>33619</v>
       </c>
@@ -1459,8 +1533,29 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I9" s="3">
+        <v>33772</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M9" s="1">
+        <v>7</v>
+      </c>
+      <c r="N9" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O9" s="2">
+        <v>8750</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>33620</v>
       </c>
@@ -1483,8 +1578,29 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I10" s="3">
+        <v>33876</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2</v>
+      </c>
+      <c r="N10" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O10" s="2">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>33623</v>
       </c>
@@ -1507,8 +1623,29 @@
         <f t="shared" si="0"/>
         <v>1120</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I11" s="3">
+        <v>34058</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M11" s="1">
+        <v>3</v>
+      </c>
+      <c r="N11" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O11" s="2">
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>33624</v>
       </c>
@@ -1531,8 +1668,29 @@
         <f t="shared" si="0"/>
         <v>2100</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I12" s="3">
+        <v>34162</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M12" s="1">
+        <v>5</v>
+      </c>
+      <c r="N12" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O12" s="2">
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>33625</v>
       </c>
@@ -1556,7 +1714,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>33626</v>
       </c>
@@ -1580,7 +1738,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>33627</v>
       </c>
@@ -1604,7 +1762,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>33628</v>
       </c>
@@ -2334,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -2344,7 +2502,7 @@
     <col min="6" max="7" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2367,7 +2525,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>33610</v>
       </c>
@@ -2391,7 +2549,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>33611</v>
       </c>
@@ -2415,7 +2573,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>33612</v>
       </c>
@@ -2439,7 +2597,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>33615</v>
       </c>
@@ -2463,7 +2621,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>33616</v>
       </c>
@@ -2486,8 +2644,17 @@
         <f t="shared" si="0"/>
         <v>4980</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>33617</v>
       </c>
@@ -2510,8 +2677,17 @@
         <f t="shared" si="0"/>
         <v>2240</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>33618</v>
       </c>
@@ -2535,7 +2711,7 @@
         <v>3750</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>33619</v>
       </c>
@@ -2558,8 +2734,29 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I9" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>33620</v>
       </c>
@@ -2582,8 +2779,29 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I10" s="3">
+        <v>33772</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M10" s="1">
+        <v>7</v>
+      </c>
+      <c r="N10" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O10" s="2">
+        <v>8750</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>33623</v>
       </c>
@@ -2606,8 +2824,29 @@
         <f t="shared" si="0"/>
         <v>1120</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I11" s="3">
+        <v>34162</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M11" s="1">
+        <v>5</v>
+      </c>
+      <c r="N11" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O11" s="2">
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>33624</v>
       </c>
@@ -2631,7 +2870,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>33625</v>
       </c>
@@ -2655,7 +2894,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>33626</v>
       </c>
@@ -2679,7 +2918,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>33627</v>
       </c>
@@ -2703,7 +2942,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>33628</v>
       </c>
@@ -3433,7 +3672,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -3443,7 +3682,7 @@
     <col min="6" max="7" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3466,7 +3705,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>33610</v>
       </c>
@@ -3490,7 +3729,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>33611</v>
       </c>
@@ -3514,7 +3753,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>33612</v>
       </c>
@@ -3538,7 +3777,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>33615</v>
       </c>
@@ -3562,7 +3801,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>33616</v>
       </c>
@@ -3586,7 +3825,7 @@
         <v>4980</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>33617</v>
       </c>
@@ -3609,8 +3848,18 @@
         <f t="shared" si="0"/>
         <v>2240</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="L7" s="8"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>33618</v>
       </c>
@@ -3633,8 +3882,18 @@
         <f t="shared" si="0"/>
         <v>3750</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="11"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>33619</v>
       </c>
@@ -3657,8 +3916,16 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9" s="14"/>
+      <c r="L9" s="13"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>33620</v>
       </c>
@@ -3682,7 +3949,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>33623</v>
       </c>
@@ -3705,8 +3972,29 @@
         <f t="shared" si="0"/>
         <v>1120</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I11" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>33624</v>
       </c>
@@ -3729,8 +4017,29 @@
         <f t="shared" si="0"/>
         <v>2100</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I12" s="3">
+        <v>33615</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="M12" s="1">
+        <v>7</v>
+      </c>
+      <c r="N12" s="2">
+        <v>500</v>
+      </c>
+      <c r="O12" s="2">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>33625</v>
       </c>
@@ -3753,8 +4062,29 @@
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I13" s="3">
+        <v>33720</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M13" s="1">
+        <v>3</v>
+      </c>
+      <c r="N13" s="2">
+        <v>1500</v>
+      </c>
+      <c r="O13" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>33626</v>
       </c>
@@ -3777,8 +4107,29 @@
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I14" s="3">
+        <v>33772</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M14" s="1">
+        <v>7</v>
+      </c>
+      <c r="N14" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O14" s="2">
+        <v>8750</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>33627</v>
       </c>
@@ -3801,8 +4152,29 @@
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I15" s="3">
+        <v>33824</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M15" s="1">
+        <v>3</v>
+      </c>
+      <c r="N15" s="2">
+        <v>1500</v>
+      </c>
+      <c r="O15" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>33628</v>
       </c>
@@ -3825,8 +4197,29 @@
         <f t="shared" si="0"/>
         <v>1160</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I16" s="3">
+        <v>33928</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M16" s="1">
+        <v>1</v>
+      </c>
+      <c r="N16" s="2">
+        <v>1500</v>
+      </c>
+      <c r="O16" s="2">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>33629</v>
       </c>
@@ -3849,8 +4242,29 @@
         <f t="shared" si="0"/>
         <v>1250</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I17" s="3">
+        <v>33980</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M17" s="1">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2">
+        <v>1500</v>
+      </c>
+      <c r="O17" s="2">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>33635</v>
       </c>
@@ -3873,8 +4287,29 @@
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I18" s="3">
+        <v>34006</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M18" s="1">
+        <v>2</v>
+      </c>
+      <c r="N18" s="2">
+        <v>1500</v>
+      </c>
+      <c r="O18" s="2">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>33636</v>
       </c>
@@ -3897,8 +4332,29 @@
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I19" s="3">
+        <v>34110</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M19" s="1">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2">
+        <v>1500</v>
+      </c>
+      <c r="O19" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>33637</v>
       </c>
@@ -3921,8 +4377,29 @@
         <f t="shared" si="0"/>
         <v>2490</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I20" s="3">
+        <v>34162</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M20" s="1">
+        <v>5</v>
+      </c>
+      <c r="N20" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O20" s="2">
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>33638</v>
       </c>
@@ -3945,8 +4422,15 @@
         <f t="shared" si="0"/>
         <v>560</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I21" s="10"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>33639</v>
       </c>
@@ -3969,8 +4453,15 @@
         <f t="shared" si="0"/>
         <v>5000</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I22" s="10"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>33640</v>
       </c>
@@ -3993,8 +4484,15 @@
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I23" s="10"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>33641</v>
       </c>
@@ -4018,7 +4516,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>33642</v>
       </c>
@@ -4042,7 +4540,7 @@
         <v>2520</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>33668</v>
       </c>
@@ -4066,7 +4564,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>33694</v>
       </c>
@@ -4090,7 +4588,7 @@
         <v>4150</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>33720</v>
       </c>
@@ -4114,7 +4612,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>33746</v>
       </c>
@@ -4138,7 +4636,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>33772</v>
       </c>
@@ -4162,7 +4660,7 @@
         <v>8750</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>33798</v>
       </c>
@@ -4186,7 +4684,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>33824</v>
       </c>
@@ -4532,7 +5030,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8.77734375" bestFit="1" customWidth="1"/>
@@ -4542,7 +5040,7 @@
     <col min="6" max="7" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -4565,7 +5063,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>33610</v>
       </c>
@@ -4589,7 +5087,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>33611</v>
       </c>
@@ -4613,7 +5111,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>33612</v>
       </c>
@@ -4637,7 +5135,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>33615</v>
       </c>
@@ -4661,7 +5159,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>33616</v>
       </c>
@@ -4685,7 +5183,7 @@
         <v>4980</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>33617</v>
       </c>
@@ -4709,7 +5207,7 @@
         <v>2240</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>33618</v>
       </c>
@@ -4733,7 +5231,7 @@
         <v>3750</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>33619</v>
       </c>
@@ -4756,8 +5254,20 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>33620</v>
       </c>
@@ -4780,8 +5290,18 @@
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" s="6"/>
+      <c r="L10" s="15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>33623</v>
       </c>
@@ -4804,8 +5324,11 @@
         <f t="shared" si="0"/>
         <v>1120</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K11" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>33624</v>
       </c>
@@ -4828,8 +5351,15 @@
         <f t="shared" si="0"/>
         <v>2100</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+    </row>
+    <row r="13" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>33625</v>
       </c>
@@ -4852,8 +5382,29 @@
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I13" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>33626</v>
       </c>
@@ -4876,8 +5427,29 @@
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I14" s="3">
+        <v>33617</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M14" s="1">
+        <v>8</v>
+      </c>
+      <c r="N14" s="2">
+        <v>280</v>
+      </c>
+      <c r="O14" s="2">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>33627</v>
       </c>
@@ -4900,8 +5472,29 @@
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I15" s="3">
+        <v>33623</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M15" s="1">
+        <v>4</v>
+      </c>
+      <c r="N15" s="2">
+        <v>280</v>
+      </c>
+      <c r="O15" s="2">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>33628</v>
       </c>
@@ -4924,8 +5517,29 @@
         <f t="shared" si="0"/>
         <v>1160</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I16" s="3">
+        <v>33638</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M16" s="1">
+        <v>2</v>
+      </c>
+      <c r="N16" s="2">
+        <v>280</v>
+      </c>
+      <c r="O16" s="2">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>33629</v>
       </c>
@@ -4948,8 +5562,29 @@
         <f t="shared" si="0"/>
         <v>1250</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I17" s="3">
+        <v>33642</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M17" s="1">
+        <v>9</v>
+      </c>
+      <c r="N17" s="2">
+        <v>280</v>
+      </c>
+      <c r="O17" s="2">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>33635</v>
       </c>
@@ -4972,8 +5607,29 @@
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I18" s="3">
+        <v>33668</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M18" s="1">
+        <v>10</v>
+      </c>
+      <c r="N18" s="2">
+        <v>280</v>
+      </c>
+      <c r="O18" s="2">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>33636</v>
       </c>
@@ -4996,8 +5652,29 @@
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I19" s="3">
+        <v>33772</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M19" s="1">
+        <v>7</v>
+      </c>
+      <c r="N19" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O19" s="2">
+        <v>8750</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>33637</v>
       </c>
@@ -5020,8 +5697,29 @@
         <f t="shared" si="0"/>
         <v>2490</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I20" s="3">
+        <v>34162</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M20" s="1">
+        <v>5</v>
+      </c>
+      <c r="N20" s="2">
+        <v>1250</v>
+      </c>
+      <c r="O20" s="2">
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>33638</v>
       </c>
@@ -5045,7 +5743,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>33639</v>
       </c>
@@ -5069,7 +5767,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>33640</v>
       </c>
@@ -5093,7 +5791,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>33641</v>
       </c>
@@ -5117,7 +5815,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>33642</v>
       </c>
@@ -5141,7 +5839,7 @@
         <v>2520</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>33668</v>
       </c>
@@ -5165,7 +5863,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>33694</v>
       </c>
@@ -5189,7 +5887,7 @@
         <v>4150</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>33720</v>
       </c>
@@ -5213,7 +5911,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>33746</v>
       </c>
@@ -5237,7 +5935,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>33772</v>
       </c>
@@ -5261,7 +5959,7 @@
         <v>8750</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>33798</v>
       </c>
@@ -5285,7 +5983,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>33824</v>
       </c>

</xml_diff>